<commit_message>
Complete manuscript source data workbook
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2_MNIST_K2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2_MNIST_K16" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3_MouseDS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig4_Leukemia" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5_McFarland" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6_MDD" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig7_Runtime" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rev_Simulation_Beta" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2d_MNIST_K2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2d_MNIST_K16" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig3d_SimDiagnostics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig4c_MouseDS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig5c_Leukemia" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6j_McFarland" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig7f_MDD" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig8_Runtime" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation_BetaSeries" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -62,12 +65,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,7 +455,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,15 +477,15 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="34" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Source data underlying manuscript ARI and runtime display items, plus the revised synthetic beta-series benchmark.</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Numerical source data underlying the calculated ARI and runtime values reported in the main manuscript figures.</t>
         </is>
       </c>
     </row>
@@ -477,63 +495,281 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>ARI is unitless. SD is the standard deviation reported for the repeated analysis. Runtime values retain the units in the supplied runtime summary files.</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>ARI source</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>results/paper_ari_reference.csv, checked against the latest manuscript.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>The Fig. 2d and Figs. 4c-7f ARI sheets were checked against bcNMF.pdf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>Runtime source</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>3 Contrastive LDA/experiments/runtime/results/20260127_175051/summary_results_final.csv and companion summaries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Fig. 8 runtime values were taken from 3 Contrastive LDA/experiments/runtime/results/20260127_175051/summary_results_final.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>Simulation source</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Generated beta-series results in demo/final_primary_ari_table.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Fig. 3d values were taken from revision_new/experiments/review5_simulation/final_background5_beta_series/results/review1_q1_sim1_sim2_5class/q1_sim1_sim2_5class_extra_metrics_summary.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Each display item has a separate worksheet. The rows in every worksheet are the numerical values used to construct that display item.</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Each worksheet contains the numerical values for the named ARI or runtime display. UMAPs and heatmaps are reproduced from the released data and notebooks.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source values for the generated count-data beta-series benchmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>beta=0</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>beta=1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>beta=2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>beta=4</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>beta=8</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>beta=16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.000 +/- 0.000</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.000 +/- 0.001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.000 +/- 0.001</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.000 +/- 0.001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.000 +/- 0.001</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.000 +/- 0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cPCA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.000 +/- 0.000</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.999 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.999 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.997 +/- 0.003</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.994 +/- 0.006</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.943 +/- 0.036</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NMF</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.000 +/- 0.000</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.001 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.002 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.001 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.001 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.001 +/- 0.002</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>bcNMF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.000 +/- 0.000</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1.000 +/- 0.000</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.999 +/- 0.002</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.997 +/- 0.003</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.998 +/- 0.004</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.965 +/- 0.011</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -793,119 +1029,539 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Source values for the Mouse-DS adjusted Rand index display.</t>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Source values for Figure 3d: target-subtype ARI and retained background-class ARI in the learned target representations. Values are mean and s.d. across five simulation seeds.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Simulation</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>ARI mean</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>ARI SD</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Provenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Target subtype ARI mean</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Target subtype ARI SD</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Retained background ARI mean</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Retained background ARI SD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>PCA</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>0.0061</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Latest manuscript and repeated-analysis summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="C3" s="7" t="n">
+        <v>0.0001524798447741</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.0010065905527678</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>cPCA</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Latest manuscript and repeated-analysis summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="C4" s="7" t="n">
+        <v>0.9944096040176352</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.0060457162651862</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.0576308519840526</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0.015831835888751</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>NMF</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Latest manuscript and repeated-analysis summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="C5" s="7" t="n">
+        <v>0.000387283222584</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.0007514906858165</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>ContrastiveVI</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0.0012824306790632</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.0017951143861723</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>iNMF (LIGER)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.001547756008392</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.0021448048360605</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.9954553368266158</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0.0041618863298211</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>iNMF (contrast)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0.0015440501714957</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.0022676104788923</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.6441869627938104</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0.299600600507568</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>UINMF</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.0005874141399484</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.0013343208219846</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.9561853362540196</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0.0979725665473081</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>SMF (supervised)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.0008535777369913</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>0.001671472298319</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>cVAE</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.7109711856945239</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.3080131071210187</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.0285989990478639</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0.0333108474944798</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 1</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>bcNMF</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0.789</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Latest manuscript and repeated-analysis summary</t>
-        </is>
+      <c r="C12" s="7" t="n">
+        <v>0.9984016</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.0035741310552358</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.0142968160613396</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0.0097865108191774</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>-9.291102018872002e-05</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.0011697482108771</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.9703556734941912</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0.0151500819363818</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>cPCA</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0.9103262772808728</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.06418262735572</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.0048182229146002</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0.0014988970803606</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>NMF</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>0.0005854250627333</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.0017664259863776</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.6327082932165619</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0.0747415662432432</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>ContrastiveVI</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.9596163800690216</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.0139357892188166</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.1911850526048304</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>0.0607041396084093</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>iNMF (LIGER)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0.0010737849478797</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.0024380283657008</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.8403438579238394</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0.1217757363275503</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>iNMF (contrast)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>0.0005601790714501</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.0013948531752527</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.6080945198302772</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0.2315264355328727</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>UINMF</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>-0.0001153418916984</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.0004983296806603</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0.9332662153786392</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>0.1045521248825681</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>SMF (supervised)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.0005945308669482</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>0.0011530813331233</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>cVAE</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>0.4050647470371361</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.363754997957394</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0.0099674672558594</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>0.0101283988877893</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Simulation 2</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>bcNMF</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>0.9354412703791044</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.0259449616595379</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>0.0026329084755649</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>0.001058397220412</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -929,7 +1585,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Source values for the Leukemia adjusted Rand index display.</t>
+          <t>Source values for the Mouse-DS adjusted Rand index display.</t>
         </is>
       </c>
     </row>
@@ -962,10 +1618,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.395</v>
+        <v>0.0061</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.002</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -980,10 +1636,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.603</v>
+        <v>0.176</v>
       </c>
       <c r="C4" t="n">
-        <v>0.027</v>
+        <v>0.02</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -998,10 +1654,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.336</v>
+        <v>0.108</v>
       </c>
       <c r="C5" t="n">
-        <v>0.022</v>
+        <v>0.006</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1016,10 +1672,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.591</v>
+        <v>0.789</v>
       </c>
       <c r="C6" t="n">
-        <v>0.047</v>
+        <v>0.024</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1053,7 +1709,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Source values for the McFarland adjusted Rand index display.</t>
+          <t>Source values for the Leukemia adjusted Rand index display.</t>
         </is>
       </c>
     </row>
@@ -1086,10 +1742,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.176</v>
+        <v>0.395</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1104,10 +1760,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.212</v>
+        <v>0.603</v>
       </c>
       <c r="C4" t="n">
-        <v>0.018</v>
+        <v>0.027</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1122,10 +1778,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.058</v>
+        <v>0.336</v>
       </c>
       <c r="C5" t="n">
-        <v>0.015</v>
+        <v>0.022</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1140,10 +1796,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.621</v>
+        <v>0.591</v>
       </c>
       <c r="C6" t="n">
-        <v>0.082</v>
+        <v>0.047</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1177,7 +1833,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Source values for the MDD adjusted Rand index display.</t>
+          <t>Source values for the McFarland adjusted Rand index display.</t>
         </is>
       </c>
     </row>
@@ -1210,10 +1866,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.06619999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="C3" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1228,10 +1884,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.051</v>
+        <v>0.212</v>
       </c>
       <c r="C4" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.018</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1246,10 +1902,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0363</v>
+        <v>0.058</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004</v>
+        <v>0.015</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1264,10 +1920,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1306</v>
+        <v>0.621</v>
       </c>
       <c r="C6" t="n">
-        <v>0.015</v>
+        <v>0.082</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1284,6 +1940,130 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source values for the MDD adjusted Rand index display.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ARI mean</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ARI SD</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.06619999999999999</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Latest manuscript and repeated-analysis summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cPCA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Latest manuscript and repeated-analysis summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NMF</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Latest manuscript and repeated-analysis summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>bcNMF</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.1306</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Latest manuscript and repeated-analysis summary</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1482,9 +2262,6 @@
       <c r="H5" t="b">
         <v>1</v>
       </c>
-      <c r="I5" t="n">
-        <v/>
-      </c>
       <c r="J5" t="n">
         <v>2</v>
       </c>
@@ -1529,9 +2306,6 @@
       <c r="J6" t="n">
         <v>2</v>
       </c>
-      <c r="K6" t="n">
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1570,9 +2344,6 @@
       <c r="J7" t="n">
         <v>2</v>
       </c>
-      <c r="K7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1687,9 +2458,6 @@
       <c r="H10" t="b">
         <v>1</v>
       </c>
-      <c r="I10" t="n">
-        <v/>
-      </c>
       <c r="J10" t="n">
         <v>2</v>
       </c>
@@ -1734,9 +2502,6 @@
       <c r="J11" t="n">
         <v>2</v>
       </c>
-      <c r="K11" t="n">
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1775,9 +2540,6 @@
       <c r="J12" t="n">
         <v>2</v>
       </c>
-      <c r="K12" t="n">
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1892,9 +2654,6 @@
       <c r="H15" t="b">
         <v>1</v>
       </c>
-      <c r="I15" t="n">
-        <v/>
-      </c>
       <c r="J15" t="n">
         <v>2</v>
       </c>
@@ -1939,9 +2698,6 @@
       <c r="J16" t="n">
         <v>2</v>
       </c>
-      <c r="K16" t="n">
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1980,9 +2736,6 @@
       <c r="J17" t="n">
         <v>2</v>
       </c>
-      <c r="K17" t="n">
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2097,9 +2850,6 @@
       <c r="H20" t="b">
         <v>1</v>
       </c>
-      <c r="I20" t="n">
-        <v/>
-      </c>
       <c r="J20" t="n">
         <v>2</v>
       </c>
@@ -2144,9 +2894,6 @@
       <c r="J21" t="n">
         <v>2</v>
       </c>
-      <c r="K21" t="n">
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2185,9 +2932,6 @@
       <c r="J22" t="n">
         <v>2</v>
       </c>
-      <c r="K22" t="n">
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2302,9 +3046,6 @@
       <c r="H25" t="b">
         <v>1</v>
       </c>
-      <c r="I25" t="n">
-        <v/>
-      </c>
       <c r="J25" t="n">
         <v>2</v>
       </c>
@@ -2349,9 +3090,6 @@
       <c r="J26" t="n">
         <v>2</v>
       </c>
-      <c r="K26" t="n">
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2390,9 +3128,6 @@
       <c r="J27" t="n">
         <v>2</v>
       </c>
-      <c r="K27" t="n">
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2507,9 +3242,6 @@
       <c r="H30" t="b">
         <v>1</v>
       </c>
-      <c r="I30" t="n">
-        <v/>
-      </c>
       <c r="J30" t="n">
         <v>2</v>
       </c>
@@ -2554,9 +3286,6 @@
       <c r="J31" t="n">
         <v>2</v>
       </c>
-      <c r="K31" t="n">
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2595,9 +3324,6 @@
       <c r="J32" t="n">
         <v>2</v>
       </c>
-      <c r="K32" t="n">
-        <v/>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2712,9 +3438,6 @@
       <c r="H35" t="b">
         <v>1</v>
       </c>
-      <c r="I35" t="n">
-        <v/>
-      </c>
       <c r="J35" t="n">
         <v>2</v>
       </c>
@@ -2759,9 +3482,6 @@
       <c r="J36" t="n">
         <v>2</v>
       </c>
-      <c r="K36" t="n">
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2799,9 +3519,6 @@
       </c>
       <c r="J37" t="n">
         <v>2</v>
-      </c>
-      <c r="K37" t="n">
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -2810,222 +3527,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Source values for the generated count-data beta-series benchmark.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>beta=0</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>beta=1</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>beta=2</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>beta=4</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>beta=8</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>beta=16</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>PCA</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1.000 +/- 0.000</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0.000 +/- 0.001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0.000 +/- 0.001</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0.000 +/- 0.001</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0.000 +/- 0.001</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0.000 +/- 0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>cPCA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1.000 +/- 0.000</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>0.999 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0.999 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0.997 +/- 0.003</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0.994 +/- 0.006</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0.943 +/- 0.036</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NMF</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1.000 +/- 0.000</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>0.001 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>0.002 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.001 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>0.001 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0.001 +/- 0.002</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>bcNMF</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1.000 +/- 0.000</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1.000 +/- 0.000</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>0.999 +/- 0.002</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0.997 +/- 0.003</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>0.998 +/- 0.004</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>0.965 +/- 0.011</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>